<commit_message>
Port nativo completo do pipeline de processamento — 10 stages nativas, 1 bridge restante
Sessões 2026-04-24/25: porta todo o fluxo de dados do monolito para
subpacotes nativos. Detalhe em handoff/CHANGES_INDEX.md.

Stages nativas adicionadas:
- compute_trechos_ponto (runtime/trechos_ponto/)
- prepare_upstream_frames (fuel_properties + kibox + motec)
- build_final_table (runtime/final_table/, 15 módulos, 2200+ linhas)
- enrich_final_table_audit (runtime/uncertainty_audit/)
- run_time_diagnostics (runtime/time_diagnostics/)
- export_excel
- run_unitary_plots (runtime/unitary_plots/, 5 módulos, ~900 linhas)

Bridge restante: run_compare_iteracoes (última).

Paridade validada: lv_kpis_clean.xlsx cell-by-cell idêntico, 74/74 PNGs
presentes, 55 byte-idênticos. 260 testes unitários verdes.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/config_incertezas_rev3.xlsx
+++ b/config/config_incertezas_rev3.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="975" yWindow="240" windowWidth="21210" windowHeight="11295" tabRatio="600" firstSheet="3" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Mappings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Instruments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Reporting_Rounding" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Defaults" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Plots" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="data quality assessment" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mappings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting_Rounding" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defaults" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plots" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data quality assessment" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.28515625" customWidth="1" min="1" max="1"/>
@@ -1047,6 +1047,168 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>Pressure sensor equipment uncertainty entered as +/-2.93 kPa via Instruments sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CO_pct</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>CO_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CO_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>California Analytical Model 30 (NDIR). Moreira_R13 Tabela C1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CO2_pct</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>CO2_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CO2_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>California Analytical Model 30 (NDIR). Moreira_R13 Tabela C1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>O2_pct</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>O2_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>O2_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>California Analytical Model 30 (paramagnetico). Moreira_R13 Tabela C1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>NOx_ppm</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NOX_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>NOX_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ppm</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>California Analytical 400-HCLD (quimiluminescencia). Moreira_R13 Tabela C1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>NO_ppm</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>NO_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>NO_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ppm</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>California Analytical 400-HCLD (quimiluminescencia). Moreira_R13 Tabela C1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>THC_ppm</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>THC_mean_of_windows</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>THC_sd_of_windows</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>ppm</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>California Analytical 300M-HFID (FID). Moreira_R13 Tabela C1.</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N149"/>
+  <dimension ref="A1:N155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="68.42578125" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9376,6 +9538,294 @@
       <c r="L149" t="inlineStr">
         <is>
           <t>Sensor accuracy limit treated as rectangular distribution: +/-2.93 kPa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>CO_pct</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>CAL_Model_30_NDIR_CO</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="n">
+        <v>20</v>
+      </c>
+      <c r="F150" t="n">
+        <v>0</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
+      <c r="I150" t="n">
+        <v>0</v>
+      </c>
+      <c r="J150" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>Model 30 NDIR. acc_pct=repetibilidade 1,0%; resolution=0,1% CO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>CO2_pct</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>CAL_Model_30_NDIR_CO2</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" t="n">
+        <v>20</v>
+      </c>
+      <c r="F151" t="n">
+        <v>0</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>Model 30 NDIR. acc_pct=repetibilidade 1,0%; resolution=0,1% CO2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>O2_pct</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>CAL_Model_30_paramag_O2</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>0</v>
+      </c>
+      <c r="E152" t="n">
+        <v>25</v>
+      </c>
+      <c r="F152" t="n">
+        <v>0</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>Model 30 paramagnetico. acc_pct=repetibilidade 1,0%; resolution=0,1% O2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>NOx_ppm</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>CAL_400-HCLD_NOx</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F153" t="n">
+        <v>0</v>
+      </c>
+      <c r="G153" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
+      <c r="I153" t="n">
+        <v>0</v>
+      </c>
+      <c r="J153" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>400-HCLD CLD. acc_pct=repetibilidade 0,5%; resolution=0,01 ppm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>NO_ppm</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>CAL_400-HCLD_NO</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F154" t="n">
+        <v>0</v>
+      </c>
+      <c r="G154" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
+      <c r="I154" t="n">
+        <v>0</v>
+      </c>
+      <c r="J154" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>400-HCLD CLD. acc_pct=repetibilidade 0,5%; resolution=0,01 ppm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>THC_ppm</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>CAL_300M-HFID_THC</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>rect</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>0</v>
+      </c>
+      <c r="E155" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F155" t="n">
+        <v>0</v>
+      </c>
+      <c r="G155" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
+      <c r="I155" t="n">
+        <v>0</v>
+      </c>
+      <c r="J155" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Moreira_R13 Tab.C1</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>300M-HFID FID. acc_pct=repetibilidade 0,5%; resolution=0,01 ppm de C.</t>
         </is>
       </c>
     </row>

</xml_diff>